<commit_message>
Matrice mise à jour automatiquement (22/10/2026 11:58)
</commit_message>
<xml_diff>
--- a/matrices/MATRICE_DE_SUIVI_DES_ACTIVITES_du_22-10-26.xlsx
+++ b/matrices/MATRICE_DE_SUIVI_DES_ACTIVITES_du_22-10-26.xlsx
@@ -954,16 +954,16 @@
         <v>46305</v>
       </c>
       <c r="L4" s="26" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="M4" s="27" t="inlineStr">
         <is>
-          <t>Travaux en cours</t>
+          <t>Non démarré</t>
         </is>
       </c>
       <c r="N4" s="22" t="inlineStr">
         <is>
-          <t>Validé</t>
+          <t>Non transmis</t>
         </is>
       </c>
       <c r="O4" s="22" t="inlineStr">
@@ -1120,16 +1120,16 @@
         <v>46315</v>
       </c>
       <c r="L6" s="26" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="M6" s="27" t="inlineStr">
         <is>
-          <t>Travaux en cours</t>
+          <t>Non démarré</t>
         </is>
       </c>
       <c r="N6" s="22" t="inlineStr">
         <is>
-          <t>Validé</t>
+          <t>Non transmis</t>
         </is>
       </c>
       <c r="O6" s="22" t="inlineStr">
@@ -2783,7 +2783,7 @@
       <c r="J30" s="49" t="n"/>
       <c r="K30" s="49" t="n"/>
       <c r="L30" s="52" t="n">
-        <v>7.69</v>
+        <v>6.54</v>
       </c>
       <c r="M30" s="48" t="n"/>
       <c r="N30" s="50" t="n"/>
@@ -3434,7 +3434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3762,7 +3762,6 @@
           <t>Validé</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
           <t>INIT</t>
@@ -3771,6 +3770,156 @@
       <c r="L6" t="inlineStr">
         <is>
           <t>2026-10-22 01:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>898842688</v>
+      </c>
+      <c r="B7" s="75" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C7" t="n">
+        <v>26</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>WORODOUGOU</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>SEGUELA</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>NOUVEAU SERVICES INTERNATIONAL COTE D’IVOIRE</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Non démarré</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>INIT</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-22 10:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>898862723</v>
+      </c>
+      <c r="B8" s="75" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>BAFING</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>KORO</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>NATHA SARL</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Non démarré</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Non transmis</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Emmanuel aka</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-22 10:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>898865037</v>
+      </c>
+      <c r="B9" s="75" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>BAGOUE</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>BOUNDIALI</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>SELECT IVOIREMULTISERVICES SARL</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Non démarré</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Non transmis</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>EV</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-22 11:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Matrice mise à jour automatiquement (22/10/2026 21:40)
</commit_message>
<xml_diff>
--- a/matrices/MATRICE_DE_SUIVI_DES_ACTIVITES_du_22-10-26.xlsx
+++ b/matrices/MATRICE_DE_SUIVI_DES_ACTIVITES_du_22-10-26.xlsx
@@ -1049,11 +1049,11 @@
         </is>
       </c>
       <c r="L5" s="26" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="M5" s="27" t="inlineStr">
         <is>
-          <t>Demarrage autorisé</t>
+          <t>Travaux en cours</t>
         </is>
       </c>
       <c r="N5" s="22" t="inlineStr">
@@ -1120,16 +1120,16 @@
         <v>46315</v>
       </c>
       <c r="L6" s="26" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="M6" s="27" t="inlineStr">
         <is>
-          <t>Non démarré</t>
+          <t>Travaux en cours</t>
         </is>
       </c>
       <c r="N6" s="22" t="inlineStr">
         <is>
-          <t>Non transmis</t>
+          <t>Validé</t>
         </is>
       </c>
       <c r="O6" s="22" t="inlineStr">
@@ -1184,16 +1184,16 @@
       <c r="J7" s="23" t="n"/>
       <c r="K7" s="23" t="n"/>
       <c r="L7" s="26" t="n">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="M7" s="27" t="inlineStr">
         <is>
-          <t>Demarrage autorisé</t>
+          <t>Travaux suspendus</t>
         </is>
       </c>
       <c r="N7" s="22" t="inlineStr">
         <is>
-          <t>Transmis</t>
+          <t>Validé</t>
         </is>
       </c>
       <c r="O7" s="22" t="inlineStr">
@@ -2783,7 +2783,7 @@
       <c r="J30" s="49" t="n"/>
       <c r="K30" s="49" t="n"/>
       <c r="L30" s="52" t="n">
-        <v>6.54</v>
+        <v>12.58</v>
       </c>
       <c r="M30" s="48" t="n"/>
       <c r="N30" s="50" t="n"/>
@@ -3434,7 +3434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3811,7 +3811,6 @@
           <t>Validé</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>INIT</t>
@@ -3861,7 +3860,6 @@
           <t>Non transmis</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>Emmanuel aka</t>
@@ -3911,7 +3909,6 @@
           <t>Non transmis</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>EV</t>
@@ -3920,6 +3917,406 @@
       <c r="L9" t="inlineStr">
         <is>
           <t>2026-10-22 11:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>899184631</v>
+      </c>
+      <c r="B10" s="75" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>BAFING</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>KORO</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>NATHA SARL</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Travaux achevés</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>100</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Transmis en cours de validation</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>KOUADIO</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-22 18:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>899185737</v>
+      </c>
+      <c r="B11" s="75" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>BAGOUE</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>BOUNDIALI</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>SELECT IVOIREMULTISERVICES SARL</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Travaux en cours</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>40</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>KOUADIO</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-22 18:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>899186054</v>
+      </c>
+      <c r="B12" s="75" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>BAFING</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>TOUBA / OUANINOU</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>SIMAGE</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Travaux en cours</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>25</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emmanuel AKA </t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-22 18:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>899186064</v>
+      </c>
+      <c r="B13" s="75" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C13" t="n">
+        <v>4</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>BAGOUE</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>KOUTO</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>IM-BTP POLYTECHNOLOGIES</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Non démarré</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Non transmis</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emmanuel AKA </t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-10-22 18:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>899192358</v>
+      </c>
+      <c r="B14" s="75" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>BAFING</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>KORO</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>NATHA SARL</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Non démarré</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Non transmis</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>KOUADIO</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-22 18:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>899193304</v>
+      </c>
+      <c r="B15" s="75" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>BAGOUE</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>BOUNDIALI</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>SELECT IVOIREMULTISERVICES SARL</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Travaux en cours</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>20</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Emmanuel A</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-22 18:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>899193311</v>
+      </c>
+      <c r="B16" s="75" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C16" t="n">
+        <v>4</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>BAGOUE</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>KOUTO</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>IM-BTP POLYTECHNOLOGIES</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Travaux suspendus</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>67</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Emmanuel</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-10-22 18:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>899194488</v>
+      </c>
+      <c r="B17" s="75" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>BAFING</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>TOUBA / OUANINOU</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>SIMAGE</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Travaux en cours</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>70</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>KOUADIO</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-10-22 18:33</t>
         </is>
       </c>
     </row>

</xml_diff>